<commit_message>
Point Tau-U handoff to the included-studies list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C4rYxzHaHkH4vso45fejDB
</commit_message>
<xml_diff>
--- a/纳入文献一览表.xlsx
+++ b/纳入文献一览表.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="513">
   <si>
     <t xml:space="preserve">纳入文献一览表</t>
   </si>
@@ -1515,6 +1515,42 @@
   </si>
   <si>
     <t xml:space="preserve">社交发起、回应、不当互动、社交游戏投入</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A1→B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A2→B+C </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分别比较</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">011-A</t>
@@ -6666,38 +6702,40 @@
       <c r="Q9" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="R9" s="8"/>
+      <c r="R9" s="8" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>81</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4</v>
@@ -6706,16 +6744,16 @@
         <v>75</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q10" s="9" t="s">
         <v>42</v>
@@ -6727,31 +6765,31 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>1</v>
@@ -6760,16 +6798,16 @@
         <v>75</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q11" s="9" t="s">
         <v>42</v>
@@ -6781,31 +6819,31 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>1</v>
@@ -6814,7 +6852,7 @@
         <v>75</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="N12" s="10" t="s">
         <v>39</v>
@@ -6823,7 +6861,7 @@
         <v>64</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Q12" s="9" t="s">
         <v>42</v>
@@ -6835,31 +6873,31 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>83</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>2</v>
@@ -6868,7 +6906,7 @@
         <v>75</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N13" s="10" t="s">
         <v>98</v>
@@ -6877,13 +6915,13 @@
         <v>40</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q13" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R13" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6891,31 +6929,31 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>93</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>3</v>
@@ -6924,16 +6962,16 @@
         <v>37</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O14" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Q14" s="9" t="s">
         <v>42</v>
@@ -6945,31 +6983,31 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>93</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>3</v>
@@ -6987,7 +7025,7 @@
         <v>40</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q15" s="9" t="s">
         <v>42</v>
@@ -6999,31 +7037,31 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4</v>
@@ -7035,13 +7073,13 @@
         <v>38</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="O16" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Q16" s="9" t="s">
         <v>42</v>
@@ -7053,31 +7091,31 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>57</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>85</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>3</v>
@@ -7086,22 +7124,22 @@
         <v>37</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="N17" s="10" t="s">
         <v>98</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="Q17" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R17" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7109,31 +7147,31 @@
         <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>57</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>112</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>3</v>
@@ -7142,16 +7180,16 @@
         <v>37</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="N18" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Q18" s="9" t="s">
         <v>42</v>
@@ -7163,31 +7201,31 @@
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I19" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3</v>
@@ -7196,7 +7234,7 @@
         <v>37</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="N19" s="10" t="s">
         <v>98</v>
@@ -7205,7 +7243,7 @@
         <v>64</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q19" s="9" t="s">
         <v>42</v>
@@ -7217,31 +7255,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>1</v>
@@ -7250,22 +7288,22 @@
         <v>75</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N20" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O20" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q20" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R20" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7273,31 +7311,31 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>4</v>
@@ -7306,22 +7344,22 @@
         <v>37</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O21" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q21" s="9" t="s">
         <v>53</v>
       </c>
       <c r="R21" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7329,31 +7367,31 @@
         <v>21</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>46</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>4</v>
@@ -7362,7 +7400,7 @@
         <v>37</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N22" s="10" t="s">
         <v>98</v>
@@ -7371,7 +7409,7 @@
         <v>40</v>
       </c>
       <c r="P22" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Q22" s="9" t="s">
         <v>53</v>
@@ -7383,31 +7421,31 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>81</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>2</v>
@@ -7416,7 +7454,7 @@
         <v>75</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N23" s="10" t="s">
         <v>77</v>
@@ -7425,13 +7463,13 @@
         <v>40</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="Q23" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R23" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7439,31 +7477,31 @@
         <v>23</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>81</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="K24" s="7" t="n">
         <v>3</v>
@@ -7472,7 +7510,7 @@
         <v>37</v>
       </c>
       <c r="M24" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N24" s="10" t="s">
         <v>39</v>
@@ -7481,7 +7519,7 @@
         <v>40</v>
       </c>
       <c r="P24" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q24" s="9" t="s">
         <v>42</v>
@@ -7493,31 +7531,31 @@
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K25" s="7" t="n">
         <v>1</v>
@@ -7526,22 +7564,22 @@
         <v>37</v>
       </c>
       <c r="M25" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O25" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q25" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R25" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7549,31 +7587,31 @@
         <v>25</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>57</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K26" s="7" t="n">
         <v>5</v>
@@ -7582,16 +7620,16 @@
         <v>75</v>
       </c>
       <c r="M26" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="N26" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O26" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P26" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q26" s="9" t="s">
         <v>42</v>
@@ -7603,31 +7641,31 @@
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K27" s="7" t="n">
         <v>2</v>
@@ -7636,7 +7674,7 @@
         <v>75</v>
       </c>
       <c r="M27" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="N27" s="10" t="s">
         <v>98</v>
@@ -7645,7 +7683,7 @@
         <v>40</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Q27" s="9" t="s">
         <v>42</v>
@@ -7657,31 +7695,31 @@
         <v>27</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>3</v>
@@ -7690,16 +7728,16 @@
         <v>37</v>
       </c>
       <c r="M28" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="N28" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O28" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P28" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q28" s="9" t="s">
         <v>42</v>
@@ -7711,31 +7749,31 @@
         <v>28</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>57</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I29" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>3</v>
@@ -7744,16 +7782,16 @@
         <v>75</v>
       </c>
       <c r="M29" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="O29" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Q29" s="9" t="s">
         <v>53</v>
@@ -7765,31 +7803,31 @@
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>81</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J30" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K30" s="7" t="n">
         <v>6</v>
@@ -7798,7 +7836,7 @@
         <v>75</v>
       </c>
       <c r="M30" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N30" s="10" t="s">
         <v>77</v>
@@ -7807,13 +7845,13 @@
         <v>64</v>
       </c>
       <c r="P30" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="Q30" s="9" t="s">
         <v>53</v>
       </c>
       <c r="R30" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7821,31 +7859,31 @@
         <v>30</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K31" s="7" t="n">
         <v>1</v>
@@ -7854,16 +7892,16 @@
         <v>75</v>
       </c>
       <c r="M31" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="Q31" s="9" t="s">
         <v>42</v>
@@ -7875,31 +7913,31 @@
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K32" s="7" t="n">
         <v>1</v>
@@ -7908,7 +7946,7 @@
         <v>37</v>
       </c>
       <c r="M32" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="N32" s="10" t="s">
         <v>98</v>
@@ -7917,13 +7955,13 @@
         <v>40</v>
       </c>
       <c r="P32" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q32" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R32" s="8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7931,31 +7969,31 @@
         <v>32</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K33" s="7" t="n">
         <v>1</v>
@@ -7964,16 +8002,16 @@
         <v>37</v>
       </c>
       <c r="M33" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="N33" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O33" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="Q33" s="9" t="s">
         <v>42</v>
@@ -7985,31 +8023,31 @@
         <v>33</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K34" s="7" t="n">
         <v>4</v>
@@ -8018,16 +8056,16 @@
         <v>75</v>
       </c>
       <c r="M34" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="N34" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O34" s="10" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="P34" s="10" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q34" s="9" t="s">
         <v>42</v>
@@ -8039,29 +8077,29 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="H35" s="8"/>
       <c r="I35" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K35" s="7" t="n">
         <v>3</v>
@@ -8070,16 +8108,16 @@
         <v>75</v>
       </c>
       <c r="M35" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O35" s="10" t="s">
         <v>40</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="Q35" s="9" t="s">
         <v>42</v>
@@ -8091,31 +8129,31 @@
         <v>35</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K36" s="7" t="n">
         <v>4</v>
@@ -8124,7 +8162,7 @@
         <v>37</v>
       </c>
       <c r="M36" s="10" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="N36" s="10" t="s">
         <v>98</v>
@@ -8133,7 +8171,7 @@
         <v>40</v>
       </c>
       <c r="P36" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Q36" s="9" t="s">
         <v>53</v>
@@ -8145,31 +8183,31 @@
         <v>36</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J37" s="8" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K37" s="7" t="n">
         <v>1</v>
@@ -8178,7 +8216,7 @@
         <v>75</v>
       </c>
       <c r="M37" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N37" s="10" t="s">
         <v>77</v>
@@ -8187,7 +8225,7 @@
         <v>40</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q37" s="9" t="s">
         <v>42</v>
@@ -8199,31 +8237,31 @@
         <v>37</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>33</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K38" s="7" t="n">
         <v>3</v>
@@ -8232,22 +8270,22 @@
         <v>75</v>
       </c>
       <c r="M38" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="N38" s="10" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="O38" s="10" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="P38" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="Q38" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R38" s="8" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8255,31 +8293,31 @@
         <v>38</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K39" s="7" t="n">
         <v>4</v>
@@ -8288,22 +8326,22 @@
         <v>37</v>
       </c>
       <c r="M39" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O39" s="10" t="s">
         <v>64</v>
       </c>
       <c r="P39" s="10" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="Q39" s="9" t="s">
         <v>53</v>
       </c>
       <c r="R39" s="10" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8311,31 +8349,31 @@
         <v>39</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K40" s="7" t="n">
         <v>3</v>
@@ -8344,16 +8382,16 @@
         <v>75</v>
       </c>
       <c r="M40" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="N40" s="10" t="s">
         <v>39</v>
       </c>
       <c r="O40" s="10" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="P40" s="10" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="Q40" s="9" t="s">
         <v>42</v>
@@ -8365,31 +8403,31 @@
         <v>40</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="I41" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K41" s="7" t="n">
         <v>3</v>
@@ -8401,13 +8439,13 @@
         <v>38</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>64</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Q41" s="9" t="s">
         <v>53</v>
@@ -8419,31 +8457,31 @@
         <v>41</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="I42" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K42" s="7" t="n">
         <v>3</v>
@@ -8461,7 +8499,7 @@
         <v>40</v>
       </c>
       <c r="P42" s="10" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="Q42" s="9" t="s">
         <v>42</v>
@@ -8473,31 +8511,31 @@
         <v>42</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J43" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="K43" s="7" t="n">
         <v>4</v>
@@ -8506,7 +8544,7 @@
         <v>37</v>
       </c>
       <c r="M43" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="N43" s="10" t="s">
         <v>98</v>
@@ -8515,13 +8553,13 @@
         <v>40</v>
       </c>
       <c r="P43" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="Q43" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R43" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8529,31 +8567,31 @@
         <v>43</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I44" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>3</v>
@@ -8568,16 +8606,16 @@
         <v>39</v>
       </c>
       <c r="O44" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="P44" s="10" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q44" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R44" s="10" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8585,31 +8623,31 @@
         <v>44</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K45" s="7" t="n">
         <v>1</v>
@@ -8618,7 +8656,7 @@
         <v>75</v>
       </c>
       <c r="M45" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="N45" s="10" t="s">
         <v>98</v>
@@ -8627,7 +8665,7 @@
         <v>40</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="Q45" s="9" t="s">
         <v>53</v>
@@ -8639,31 +8677,31 @@
         <v>45</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>73</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K46" s="7" t="n">
         <v>3</v>
@@ -8672,7 +8710,7 @@
         <v>75</v>
       </c>
       <c r="M46" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="N46" s="10" t="s">
         <v>77</v>
@@ -8681,7 +8719,7 @@
         <v>106</v>
       </c>
       <c r="P46" s="10" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="Q46" s="9" t="s">
         <v>53</v>
@@ -8693,29 +8731,29 @@
         <v>46</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="H47" s="8"/>
       <c r="I47" s="10" t="s">
         <v>85</v>
       </c>
       <c r="J47" s="10" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K47" s="7" t="n">
         <v>3</v>
@@ -8724,27 +8762,27 @@
         <v>37</v>
       </c>
       <c r="M47" s="10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N47" s="10" t="s">
         <v>98</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="Q47" s="9" t="s">
         <v>42</v>
       </c>
       <c r="R47" s="10" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J49" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K49" s="11" t="n">
         <f aca="false">SUM(K2:K47)</f>
@@ -8753,7 +8791,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J50" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K50" s="11" t="n">
         <f aca="false">COUNTA(B2:B47)</f>
@@ -8762,7 +8800,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
   </sheetData>
@@ -8831,16 +8869,16 @@
         <v>18</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="N1" s="6" t="s">
         <v>26</v>
@@ -8854,40 +8892,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="N2" s="9" t="s">
         <v>53</v>
@@ -8899,46 +8937,46 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>46</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="N3" s="9" t="s">
         <v>53</v>
       </c>
       <c r="O3" s="10" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8946,46 +8984,46 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="N4" s="9" t="s">
         <v>42</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8993,40 +9031,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>46</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="N5" s="9" t="s">
         <v>53</v>
@@ -9038,44 +9076,44 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="10" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="N6" s="9" t="s">
         <v>53</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>